<commit_message>
feat: implementacion PRD v3.5.0 con roles, brecha no-sabe, TDR HSA y portal admin
</commit_message>
<xml_diff>
--- a/Registro_General_ProtegeDatosLocal.xlsx
+++ b/Registro_General_ProtegeDatosLocal.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -571,56 +571,6 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Vía de Contratación</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>23-08-2026 03:18:42</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>I. Municipalidad de Santiago</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Auditor Ético</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>CISO</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>auditoria.final@chile.cl</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>SECPLA_TI</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo / Diagnóstico Iniciado</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>Remitir Informe Ejecutivo y TDR en Word</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Honorarios Suma Alzada (Art. 4 Ley 18.883)</t>
         </is>
       </c>
     </row>

</xml_diff>